<commit_message>
changes made ot template
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000" firstSheet="1"/>
+    <workbookView windowWidth="23040" windowHeight="8280" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="template" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="337" uniqueCount="177">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -54,6 +54,15 @@
     <t>Priority</t>
   </si>
   <si>
+    <t>Execution Status</t>
+  </si>
+  <si>
+    <t>Bug Status</t>
+  </si>
+  <si>
+    <t>Bug ID</t>
+  </si>
+  <si>
     <t>Functional Test Cases</t>
   </si>
   <si>
@@ -67,6 +76,9 @@
   </si>
   <si>
     <t>Critical</t>
+  </si>
+  <si>
+    <t>Pass</t>
   </si>
   <si>
     <t>FT-02</t>
@@ -941,7 +953,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="21">
     <border>
       <left/>
       <right/>
@@ -1088,6 +1100,19 @@
     </border>
     <border>
       <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
       <right style="thin">
@@ -1208,7 +1233,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="12" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="13" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1220,34 +1245,34 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="15" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="16" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="17" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="18" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="19" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1332,7 +1357,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1392,9 +1417,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1404,6 +1426,17 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1743,8 +1776,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H157"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8" outlineLevelCol="7"/>
+  <dimension ref="A1:K157"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="14.575" style="2" customWidth="1"/>
     <col min="2" max="2" width="40.8583333333333" style="2" customWidth="1"/>
@@ -1754,10 +1787,13 @@
     <col min="6" max="6" width="18.7083333333333" style="2" customWidth="1"/>
     <col min="7" max="7" width="17.2833333333333" style="2" customWidth="1"/>
     <col min="8" max="8" width="12.575" style="2" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="2"/>
+    <col min="9" max="9" width="16.975" style="2" customWidth="1"/>
+    <col min="10" max="10" width="15.475" style="2" customWidth="1"/>
+    <col min="11" max="11" width="13.4166666666667" style="2" customWidth="1"/>
+    <col min="12" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" ht="27.6" spans="1:11">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -1782,10 +1818,19 @@
       <c r="H1" s="10" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" ht="14.45" customHeight="1" spans="1:8">
+      <c r="I1" s="26" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="26" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="26" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" ht="14.45" customHeight="1" spans="1:11">
       <c r="A2" s="11" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -1794,17 +1839,20 @@
       <c r="F2" s="12"/>
       <c r="G2" s="12"/>
       <c r="H2" s="13"/>
-    </row>
-    <row r="3" spans="1:8">
+      <c r="I2" s="27"/>
+      <c r="J2" s="27"/>
+      <c r="K2" s="27"/>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" s="14" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B3" s="15" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C3" s="15"/>
       <c r="D3" s="15" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E3" s="15"/>
       <c r="F3" s="15" t="s">
@@ -1812,12 +1860,17 @@
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="15" t="s">
-        <v>12</v>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="I3" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="29"/>
+      <c r="K3" s="30"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="14" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
@@ -1829,7 +1882,7 @@
     </row>
     <row r="5" spans="1:8">
       <c r="A5" s="14" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
@@ -1841,7 +1894,7 @@
     </row>
     <row r="6" spans="1:8">
       <c r="A6" s="14" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B6" s="15"/>
       <c r="C6" s="15"/>
@@ -1853,7 +1906,7 @@
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="14" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B7" s="15"/>
       <c r="C7" s="15"/>
@@ -1865,7 +1918,7 @@
     </row>
     <row r="8" spans="1:8">
       <c r="A8" s="14" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -1877,7 +1930,7 @@
     </row>
     <row r="9" spans="1:8">
       <c r="A9" s="14" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B9" s="15"/>
       <c r="C9" s="15"/>
@@ -1889,7 +1942,7 @@
     </row>
     <row r="10" spans="1:8">
       <c r="A10" s="14" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B10" s="15"/>
       <c r="C10" s="15"/>
@@ -1901,7 +1954,7 @@
     </row>
     <row r="11" spans="1:8">
       <c r="A11" s="14" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B11" s="21"/>
       <c r="C11" s="15"/>
@@ -1913,7 +1966,7 @@
     </row>
     <row r="12" spans="1:8">
       <c r="A12" s="14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
@@ -1925,7 +1978,7 @@
     </row>
     <row r="13" s="19" customFormat="1" spans="1:8">
       <c r="A13" s="14" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B13" s="21"/>
       <c r="C13" s="15"/>
@@ -1937,7 +1990,7 @@
     </row>
     <row r="14" s="19" customFormat="1" spans="1:8">
       <c r="A14" s="14" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B14" s="15"/>
       <c r="C14" s="15"/>
@@ -1949,7 +2002,7 @@
     </row>
     <row r="15" s="19" customFormat="1" spans="1:8">
       <c r="A15" s="14" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B15" s="15"/>
       <c r="C15" s="15"/>
@@ -1961,7 +2014,7 @@
     </row>
     <row r="16" s="19" customFormat="1" spans="1:8">
       <c r="A16" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B16" s="15"/>
       <c r="C16" s="15"/>
@@ -1973,7 +2026,7 @@
     </row>
     <row r="17" s="19" customFormat="1" spans="1:8">
       <c r="A17" s="14" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B17" s="15"/>
       <c r="C17" s="15"/>
@@ -1985,7 +2038,7 @@
     </row>
     <row r="18" s="19" customFormat="1" spans="1:8">
       <c r="A18" s="14" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
@@ -1997,7 +2050,7 @@
     </row>
     <row r="19" s="19" customFormat="1" spans="1:8">
       <c r="A19" s="14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B19" s="15"/>
       <c r="C19" s="15"/>
@@ -2009,7 +2062,7 @@
     </row>
     <row r="20" s="19" customFormat="1" spans="1:8">
       <c r="A20" s="14" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B20" s="15"/>
       <c r="C20" s="15"/>
@@ -2021,7 +2074,7 @@
     </row>
     <row r="21" s="19" customFormat="1" spans="1:8">
       <c r="A21" s="14" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B21" s="15"/>
       <c r="C21" s="15"/>
@@ -2033,7 +2086,7 @@
     </row>
     <row r="22" s="19" customFormat="1" spans="1:8">
       <c r="A22" s="14" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B22" s="15"/>
       <c r="C22" s="15"/>
@@ -2045,7 +2098,7 @@
     </row>
     <row r="23" s="19" customFormat="1" spans="1:8">
       <c r="A23" s="14" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B23" s="15"/>
       <c r="C23" s="15"/>
@@ -2057,7 +2110,7 @@
     </row>
     <row r="24" s="19" customFormat="1" spans="1:8">
       <c r="A24" s="14" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B24" s="15"/>
       <c r="C24" s="15"/>
@@ -2069,7 +2122,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="14" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B25" s="22"/>
       <c r="C25" s="22"/>
@@ -2081,7 +2134,7 @@
     </row>
     <row r="26" customFormat="1" spans="1:8">
       <c r="A26" s="14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B26" s="22"/>
       <c r="C26" s="22"/>
@@ -2093,7 +2146,7 @@
     </row>
     <row r="27" customFormat="1" spans="1:8">
       <c r="A27" s="14" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B27" s="22"/>
       <c r="C27" s="22"/>
@@ -2105,7 +2158,7 @@
     </row>
     <row r="28" customFormat="1" spans="1:8">
       <c r="A28" s="14" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B28" s="22"/>
       <c r="C28" s="22"/>
@@ -2117,7 +2170,7 @@
     </row>
     <row r="29" customFormat="1" spans="1:8">
       <c r="A29" s="14" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B29" s="22"/>
       <c r="C29" s="22"/>
@@ -2129,7 +2182,7 @@
     </row>
     <row r="30" customFormat="1" spans="1:8">
       <c r="A30" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B30" s="22"/>
       <c r="C30" s="22"/>
@@ -2141,7 +2194,7 @@
     </row>
     <row r="31" customFormat="1" spans="1:8">
       <c r="A31" s="14" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B31" s="22"/>
       <c r="C31" s="22"/>
@@ -2153,7 +2206,7 @@
     </row>
     <row r="32" customFormat="1" spans="1:8">
       <c r="A32" s="14" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B32" s="22"/>
       <c r="C32" s="22"/>
@@ -2165,7 +2218,7 @@
     </row>
     <row r="33" customFormat="1" spans="1:8">
       <c r="A33" s="14" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B33" s="22"/>
       <c r="C33" s="22"/>
@@ -2177,7 +2230,7 @@
     </row>
     <row r="34" customFormat="1" spans="1:8">
       <c r="A34" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B34" s="22"/>
       <c r="C34" s="22"/>
@@ -2189,7 +2242,7 @@
     </row>
     <row r="35" customFormat="1" spans="1:8">
       <c r="A35" s="14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B35" s="22"/>
       <c r="C35" s="22"/>
@@ -2201,7 +2254,7 @@
     </row>
     <row r="36" customFormat="1" spans="1:8">
       <c r="A36" s="14" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B36" s="22"/>
       <c r="C36" s="22"/>
@@ -2213,187 +2266,187 @@
     </row>
     <row r="37" customFormat="1" spans="1:8">
       <c r="A37" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B37" s="23"/>
-      <c r="C37" s="23"/>
-      <c r="D37" s="23"/>
-      <c r="E37" s="23"/>
-      <c r="F37" s="23"/>
-      <c r="G37" s="23"/>
-      <c r="H37" s="23"/>
+        <v>50</v>
+      </c>
+      <c r="B37" s="22"/>
+      <c r="C37" s="22"/>
+      <c r="D37" s="22"/>
+      <c r="E37" s="22"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
     </row>
     <row r="38" customFormat="1" spans="1:8">
       <c r="A38" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="B38" s="23"/>
-      <c r="C38" s="23"/>
-      <c r="D38" s="23"/>
-      <c r="E38" s="23"/>
-      <c r="F38" s="23"/>
-      <c r="G38" s="23"/>
-      <c r="H38" s="23"/>
+        <v>51</v>
+      </c>
+      <c r="B38" s="22"/>
+      <c r="C38" s="22"/>
+      <c r="D38" s="22"/>
+      <c r="E38" s="22"/>
+      <c r="F38" s="22"/>
+      <c r="G38" s="22"/>
+      <c r="H38" s="22"/>
     </row>
     <row r="39" customFormat="1" spans="1:8">
       <c r="A39" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B39" s="23"/>
-      <c r="C39" s="23"/>
-      <c r="D39" s="23"/>
-      <c r="E39" s="23"/>
-      <c r="F39" s="23"/>
-      <c r="G39" s="23"/>
-      <c r="H39" s="23"/>
+        <v>52</v>
+      </c>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="22"/>
+      <c r="H39" s="22"/>
     </row>
     <row r="40" customFormat="1" spans="1:8">
       <c r="A40" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B40" s="23"/>
-      <c r="C40" s="23"/>
-      <c r="D40" s="23"/>
-      <c r="E40" s="23"/>
-      <c r="F40" s="23"/>
-      <c r="G40" s="23"/>
-      <c r="H40" s="23"/>
+        <v>53</v>
+      </c>
+      <c r="B40" s="22"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
+      <c r="E40" s="22"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="22"/>
+      <c r="H40" s="22"/>
     </row>
     <row r="41" customFormat="1" spans="1:8">
       <c r="A41" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="B41" s="23"/>
-      <c r="C41" s="23"/>
-      <c r="D41" s="23"/>
-      <c r="E41" s="23"/>
-      <c r="F41" s="23"/>
-      <c r="G41" s="23"/>
-      <c r="H41" s="23"/>
+        <v>54</v>
+      </c>
+      <c r="B41" s="22"/>
+      <c r="C41" s="22"/>
+      <c r="D41" s="22"/>
+      <c r="E41" s="22"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="22"/>
     </row>
     <row r="42" customFormat="1" spans="1:8">
       <c r="A42" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="B42" s="23"/>
-      <c r="C42" s="23"/>
-      <c r="D42" s="23"/>
-      <c r="E42" s="23"/>
-      <c r="F42" s="23"/>
-      <c r="G42" s="23"/>
-      <c r="H42" s="23"/>
+        <v>55</v>
+      </c>
+      <c r="B42" s="22"/>
+      <c r="C42" s="22"/>
+      <c r="D42" s="22"/>
+      <c r="E42" s="22"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="22"/>
+      <c r="H42" s="22"/>
     </row>
     <row r="43" customFormat="1" spans="1:8">
       <c r="A43" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="B43" s="23"/>
-      <c r="C43" s="23"/>
-      <c r="D43" s="23"/>
-      <c r="E43" s="23"/>
-      <c r="F43" s="23"/>
-      <c r="G43" s="23"/>
-      <c r="H43" s="23"/>
+        <v>56</v>
+      </c>
+      <c r="B43" s="22"/>
+      <c r="C43" s="22"/>
+      <c r="D43" s="22"/>
+      <c r="E43" s="22"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="22"/>
     </row>
     <row r="44" customFormat="1" spans="1:8">
       <c r="A44" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B44" s="23"/>
-      <c r="C44" s="23"/>
-      <c r="D44" s="23"/>
-      <c r="E44" s="23"/>
-      <c r="F44" s="23"/>
-      <c r="G44" s="23"/>
-      <c r="H44" s="23"/>
+        <v>57</v>
+      </c>
+      <c r="B44" s="22"/>
+      <c r="C44" s="22"/>
+      <c r="D44" s="22"/>
+      <c r="E44" s="22"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="22"/>
+      <c r="H44" s="22"/>
     </row>
     <row r="45" customFormat="1" spans="1:8">
       <c r="A45" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B45" s="23"/>
-      <c r="C45" s="23"/>
-      <c r="D45" s="23"/>
-      <c r="E45" s="23"/>
-      <c r="F45" s="23"/>
-      <c r="G45" s="23"/>
-      <c r="H45" s="23"/>
+        <v>58</v>
+      </c>
+      <c r="B45" s="22"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
+      <c r="E45" s="22"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="22"/>
+      <c r="H45" s="22"/>
     </row>
     <row r="46" customFormat="1" spans="1:8">
       <c r="A46" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B46" s="23"/>
-      <c r="C46" s="23"/>
-      <c r="D46" s="23"/>
-      <c r="E46" s="23"/>
-      <c r="F46" s="23"/>
-      <c r="G46" s="23"/>
-      <c r="H46" s="23"/>
+        <v>59</v>
+      </c>
+      <c r="B46" s="22"/>
+      <c r="C46" s="22"/>
+      <c r="D46" s="22"/>
+      <c r="E46" s="22"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="22"/>
     </row>
     <row r="47" customFormat="1" spans="1:8">
       <c r="A47" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="B47" s="23"/>
-      <c r="C47" s="23"/>
-      <c r="D47" s="23"/>
-      <c r="E47" s="23"/>
-      <c r="F47" s="23"/>
-      <c r="G47" s="23"/>
-      <c r="H47" s="23"/>
+        <v>60</v>
+      </c>
+      <c r="B47" s="22"/>
+      <c r="C47" s="22"/>
+      <c r="D47" s="22"/>
+      <c r="E47" s="22"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
+      <c r="H47" s="22"/>
     </row>
     <row r="48" customFormat="1" spans="1:8">
       <c r="A48" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="B48" s="23"/>
-      <c r="C48" s="23"/>
-      <c r="D48" s="23"/>
-      <c r="E48" s="23"/>
-      <c r="F48" s="23"/>
-      <c r="G48" s="23"/>
-      <c r="H48" s="23"/>
+        <v>61</v>
+      </c>
+      <c r="B48" s="22"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="22"/>
+      <c r="H48" s="22"/>
     </row>
     <row r="49" customFormat="1" spans="1:8">
       <c r="A49" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="B49" s="23"/>
-      <c r="C49" s="23"/>
-      <c r="D49" s="23"/>
-      <c r="E49" s="23"/>
-      <c r="F49" s="23"/>
-      <c r="G49" s="23"/>
-      <c r="H49" s="23"/>
+        <v>62</v>
+      </c>
+      <c r="B49" s="22"/>
+      <c r="C49" s="22"/>
+      <c r="D49" s="22"/>
+      <c r="E49" s="22"/>
+      <c r="F49" s="22"/>
+      <c r="G49" s="22"/>
+      <c r="H49" s="22"/>
     </row>
     <row r="50" customFormat="1" spans="1:8">
       <c r="A50" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B50" s="23"/>
-      <c r="C50" s="23"/>
-      <c r="D50" s="23"/>
-      <c r="E50" s="23"/>
-      <c r="F50" s="23"/>
-      <c r="G50" s="23"/>
-      <c r="H50" s="23"/>
+        <v>63</v>
+      </c>
+      <c r="B50" s="22"/>
+      <c r="C50" s="22"/>
+      <c r="D50" s="22"/>
+      <c r="E50" s="22"/>
+      <c r="F50" s="22"/>
+      <c r="G50" s="22"/>
+      <c r="H50" s="22"/>
     </row>
     <row r="51" customFormat="1" spans="1:8">
       <c r="A51" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B51" s="23"/>
-      <c r="C51" s="23"/>
-      <c r="D51" s="23"/>
-      <c r="E51" s="23"/>
-      <c r="F51" s="23"/>
-      <c r="G51" s="23"/>
-      <c r="H51" s="23"/>
+        <v>64</v>
+      </c>
+      <c r="B51" s="22"/>
+      <c r="C51" s="22"/>
+      <c r="D51" s="22"/>
+      <c r="E51" s="22"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="22"/>
+      <c r="H51" s="22"/>
     </row>
     <row r="52" s="20" customFormat="1" spans="1:8">
       <c r="A52" s="14" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B52" s="15"/>
       <c r="C52" s="15"/>
@@ -2404,20 +2457,20 @@
       <c r="H52" s="15"/>
     </row>
     <row r="53" s="1" customFormat="1" ht="14.45" customHeight="1" spans="1:8">
-      <c r="A53" s="24" t="s">
-        <v>62</v>
-      </c>
-      <c r="B53" s="25"/>
-      <c r="C53" s="25"/>
-      <c r="D53" s="25"/>
-      <c r="E53" s="25"/>
-      <c r="F53" s="25"/>
-      <c r="G53" s="25"/>
-      <c r="H53" s="26"/>
+      <c r="A53" s="23" t="s">
+        <v>66</v>
+      </c>
+      <c r="B53" s="24"/>
+      <c r="C53" s="24"/>
+      <c r="D53" s="24"/>
+      <c r="E53" s="24"/>
+      <c r="F53" s="24"/>
+      <c r="G53" s="24"/>
+      <c r="H53" s="25"/>
     </row>
     <row r="54" s="2" customFormat="1" spans="1:8">
       <c r="A54" s="14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B54" s="15"/>
       <c r="C54" s="15"/>
@@ -2429,7 +2482,7 @@
     </row>
     <row r="55" s="2" customFormat="1" spans="1:8">
       <c r="A55" s="14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B55" s="15"/>
       <c r="C55" s="15"/>
@@ -2441,7 +2494,7 @@
     </row>
     <row r="56" s="2" customFormat="1" spans="1:8">
       <c r="A56" s="14" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B56" s="15"/>
       <c r="C56" s="15"/>
@@ -2453,7 +2506,7 @@
     </row>
     <row r="57" s="2" customFormat="1" spans="1:8">
       <c r="A57" s="14" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B57" s="15"/>
       <c r="C57" s="15"/>
@@ -2465,7 +2518,7 @@
     </row>
     <row r="58" s="2" customFormat="1" spans="1:8">
       <c r="A58" s="14" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B58" s="15"/>
       <c r="C58" s="15"/>
@@ -2477,7 +2530,7 @@
     </row>
     <row r="59" s="2" customFormat="1" spans="1:8">
       <c r="A59" s="14" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B59" s="15"/>
       <c r="C59" s="15"/>
@@ -2489,7 +2542,7 @@
     </row>
     <row r="60" s="2" customFormat="1" spans="1:8">
       <c r="A60" s="14" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B60" s="15"/>
       <c r="C60" s="15"/>
@@ -2501,7 +2554,7 @@
     </row>
     <row r="61" s="2" customFormat="1" spans="1:8">
       <c r="A61" s="14" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B61" s="15"/>
       <c r="C61" s="15"/>
@@ -2513,7 +2566,7 @@
     </row>
     <row r="62" s="2" customFormat="1" spans="1:8">
       <c r="A62" s="14" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B62" s="15"/>
       <c r="C62" s="15"/>
@@ -2525,7 +2578,7 @@
     </row>
     <row r="63" s="2" customFormat="1" spans="1:8">
       <c r="A63" s="14" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B63" s="15"/>
       <c r="C63" s="15"/>
@@ -2537,7 +2590,7 @@
     </row>
     <row r="64" s="2" customFormat="1" spans="1:8">
       <c r="A64" s="14" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B64" s="15"/>
       <c r="C64" s="15"/>
@@ -2549,7 +2602,7 @@
     </row>
     <row r="65" s="2" customFormat="1" spans="1:8">
       <c r="A65" s="14" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B65" s="15"/>
       <c r="C65" s="15"/>
@@ -2561,7 +2614,7 @@
     </row>
     <row r="66" s="2" customFormat="1" spans="1:8">
       <c r="A66" s="14" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B66" s="15"/>
       <c r="C66" s="15"/>
@@ -2573,7 +2626,7 @@
     </row>
     <row r="67" s="2" customFormat="1" spans="1:8">
       <c r="A67" s="14" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B67" s="15"/>
       <c r="C67" s="15"/>
@@ -2585,7 +2638,7 @@
     </row>
     <row r="68" s="2" customFormat="1" spans="1:8">
       <c r="A68" s="14" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B68" s="15"/>
       <c r="C68" s="15"/>
@@ -2597,7 +2650,7 @@
     </row>
     <row r="69" s="2" customFormat="1" spans="1:8">
       <c r="A69" s="14" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B69" s="15"/>
       <c r="C69" s="15"/>
@@ -2609,7 +2662,7 @@
     </row>
     <row r="70" s="2" customFormat="1" spans="1:8">
       <c r="A70" s="14" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B70" s="15"/>
       <c r="C70" s="15"/>
@@ -2621,7 +2674,7 @@
     </row>
     <row r="71" s="2" customFormat="1" spans="1:8">
       <c r="A71" s="14" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B71" s="15"/>
       <c r="C71" s="15"/>
@@ -2633,7 +2686,7 @@
     </row>
     <row r="72" s="2" customFormat="1" spans="1:8">
       <c r="A72" s="14" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B72" s="15"/>
       <c r="C72" s="15"/>
@@ -2645,7 +2698,7 @@
     </row>
     <row r="73" s="2" customFormat="1" spans="1:8">
       <c r="A73" s="14" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B73" s="15"/>
       <c r="C73" s="15"/>
@@ -2657,7 +2710,7 @@
     </row>
     <row r="74" s="1" customFormat="1" ht="14.45" customHeight="1" spans="1:8">
       <c r="A74" s="11" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B74" s="12"/>
       <c r="C74" s="12"/>
@@ -2669,7 +2722,7 @@
     </row>
     <row r="75" s="2" customFormat="1" spans="1:8">
       <c r="A75" s="14" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B75" s="15"/>
       <c r="C75" s="15"/>
@@ -2681,7 +2734,7 @@
     </row>
     <row r="76" s="2" customFormat="1" spans="1:8">
       <c r="A76" s="14" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B76" s="15"/>
       <c r="C76" s="15"/>
@@ -2693,7 +2746,7 @@
     </row>
     <row r="77" s="2" customFormat="1" spans="1:8">
       <c r="A77" s="14" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B77" s="15"/>
       <c r="C77" s="15"/>
@@ -2705,7 +2758,7 @@
     </row>
     <row r="78" s="2" customFormat="1" spans="1:8">
       <c r="A78" s="14" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B78" s="15"/>
       <c r="C78" s="15"/>
@@ -2717,7 +2770,7 @@
     </row>
     <row r="79" s="2" customFormat="1" spans="1:8">
       <c r="A79" s="14" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B79" s="15"/>
       <c r="C79" s="15"/>
@@ -2729,7 +2782,7 @@
     </row>
     <row r="80" s="2" customFormat="1" spans="1:8">
       <c r="A80" s="14" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B80" s="15"/>
       <c r="C80" s="15"/>
@@ -2741,7 +2794,7 @@
     </row>
     <row r="81" s="2" customFormat="1" spans="1:8">
       <c r="A81" s="14" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B81" s="15"/>
       <c r="C81" s="15"/>
@@ -2753,7 +2806,7 @@
     </row>
     <row r="82" s="2" customFormat="1" spans="1:8">
       <c r="A82" s="14" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B82" s="15"/>
       <c r="C82" s="15"/>
@@ -2765,7 +2818,7 @@
     </row>
     <row r="83" s="2" customFormat="1" spans="1:8">
       <c r="A83" s="14" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B83" s="15"/>
       <c r="C83" s="15"/>
@@ -2777,7 +2830,7 @@
     </row>
     <row r="84" s="2" customFormat="1" spans="1:8">
       <c r="A84" s="14" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B84" s="15"/>
       <c r="C84" s="15"/>
@@ -2789,7 +2842,7 @@
     </row>
     <row r="85" s="2" customFormat="1" spans="1:8">
       <c r="A85" s="14" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B85" s="15"/>
       <c r="C85" s="15"/>
@@ -2801,7 +2854,7 @@
     </row>
     <row r="86" s="2" customFormat="1" spans="1:8">
       <c r="A86" s="14" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B86" s="15"/>
       <c r="C86" s="15"/>
@@ -2813,7 +2866,7 @@
     </row>
     <row r="87" s="2" customFormat="1" spans="1:8">
       <c r="A87" s="14" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B87" s="15"/>
       <c r="C87" s="15"/>
@@ -2825,7 +2878,7 @@
     </row>
     <row r="88" s="2" customFormat="1" spans="1:8">
       <c r="A88" s="14" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B88" s="15"/>
       <c r="C88" s="15"/>
@@ -2837,7 +2890,7 @@
     </row>
     <row r="89" s="2" customFormat="1" spans="1:8">
       <c r="A89" s="14" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B89" s="15"/>
       <c r="C89" s="15"/>
@@ -2849,7 +2902,7 @@
     </row>
     <row r="90" s="2" customFormat="1" spans="1:8">
       <c r="A90" s="14" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B90" s="15"/>
       <c r="C90" s="15"/>
@@ -2861,7 +2914,7 @@
     </row>
     <row r="91" s="2" customFormat="1" spans="1:8">
       <c r="A91" s="14" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B91" s="15"/>
       <c r="C91" s="15"/>
@@ -2873,7 +2926,7 @@
     </row>
     <row r="92" s="2" customFormat="1" spans="1:8">
       <c r="A92" s="14" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B92" s="15"/>
       <c r="C92" s="15"/>
@@ -2885,7 +2938,7 @@
     </row>
     <row r="93" s="2" customFormat="1" spans="1:8">
       <c r="A93" s="14" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B93" s="15"/>
       <c r="C93" s="15"/>
@@ -2897,7 +2950,7 @@
     </row>
     <row r="94" s="2" customFormat="1" spans="1:8">
       <c r="A94" s="14" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B94" s="15"/>
       <c r="C94" s="15"/>
@@ -2909,7 +2962,7 @@
     </row>
     <row r="95" ht="14.45" customHeight="1" spans="1:8">
       <c r="A95" s="11" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B95" s="12"/>
       <c r="C95" s="12"/>
@@ -2921,7 +2974,7 @@
     </row>
     <row r="96" spans="1:8">
       <c r="A96" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B96" s="15"/>
       <c r="C96" s="15"/>
@@ -2933,7 +2986,7 @@
     </row>
     <row r="97" spans="1:8">
       <c r="A97" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B97" s="15"/>
       <c r="C97" s="15"/>
@@ -2945,7 +2998,7 @@
     </row>
     <row r="98" spans="1:8">
       <c r="A98" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B98" s="15"/>
       <c r="C98" s="15"/>
@@ -2957,7 +3010,7 @@
     </row>
     <row r="99" spans="1:8">
       <c r="A99" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B99" s="15"/>
       <c r="C99" s="15"/>
@@ -2969,7 +3022,7 @@
     </row>
     <row r="100" spans="1:8">
       <c r="A100" s="14" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B100" s="15"/>
       <c r="C100" s="15"/>
@@ -2981,7 +3034,7 @@
     </row>
     <row r="101" spans="1:8">
       <c r="A101" s="14" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B101" s="15"/>
       <c r="C101" s="15"/>
@@ -2993,7 +3046,7 @@
     </row>
     <row r="102" spans="1:8">
       <c r="A102" s="14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B102" s="15"/>
       <c r="C102" s="15"/>
@@ -3005,7 +3058,7 @@
     </row>
     <row r="103" spans="1:8">
       <c r="A103" s="14" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B103" s="15"/>
       <c r="C103" s="15"/>
@@ -3017,7 +3070,7 @@
     </row>
     <row r="104" spans="1:8">
       <c r="A104" s="14" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B104" s="15"/>
       <c r="C104" s="15"/>
@@ -3029,7 +3082,7 @@
     </row>
     <row r="105" spans="1:8">
       <c r="A105" s="14" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B105" s="15"/>
       <c r="C105" s="15"/>
@@ -3041,7 +3094,7 @@
     </row>
     <row r="106" spans="1:8">
       <c r="A106" s="14" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
@@ -3053,7 +3106,7 @@
     </row>
     <row r="107" spans="1:8">
       <c r="A107" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B107" s="15"/>
       <c r="C107" s="15"/>
@@ -3065,7 +3118,7 @@
     </row>
     <row r="108" spans="1:8">
       <c r="A108" s="14" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
@@ -3077,7 +3130,7 @@
     </row>
     <row r="109" spans="1:8">
       <c r="A109" s="14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B109" s="15"/>
       <c r="C109" s="15"/>
@@ -3089,7 +3142,7 @@
     </row>
     <row r="110" spans="1:8">
       <c r="A110" s="14" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B110" s="15"/>
       <c r="C110" s="15"/>
@@ -3101,7 +3154,7 @@
     </row>
     <row r="111" spans="1:8">
       <c r="A111" s="14" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B111" s="15"/>
       <c r="C111" s="15"/>
@@ -3113,7 +3166,7 @@
     </row>
     <row r="112" spans="1:8">
       <c r="A112" s="14" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
@@ -3125,7 +3178,7 @@
     </row>
     <row r="113" spans="1:8">
       <c r="A113" s="14" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B113" s="15"/>
       <c r="C113" s="15"/>
@@ -3137,7 +3190,7 @@
     </row>
     <row r="114" spans="1:8">
       <c r="A114" s="14" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
@@ -3149,7 +3202,7 @@
     </row>
     <row r="115" spans="1:8">
       <c r="A115" s="14" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
@@ -3161,7 +3214,7 @@
     </row>
     <row r="116" ht="14.45" customHeight="1" spans="1:8">
       <c r="A116" s="11" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B116" s="12"/>
       <c r="C116" s="12"/>
@@ -3173,7 +3226,7 @@
     </row>
     <row r="117" spans="1:8">
       <c r="A117" s="14" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
@@ -3185,7 +3238,7 @@
     </row>
     <row r="118" spans="1:8">
       <c r="A118" s="14" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
@@ -3197,7 +3250,7 @@
     </row>
     <row r="119" spans="1:8">
       <c r="A119" s="14" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
@@ -3209,7 +3262,7 @@
     </row>
     <row r="120" spans="1:8">
       <c r="A120" s="14" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
@@ -3221,7 +3274,7 @@
     </row>
     <row r="121" spans="1:8">
       <c r="A121" s="14" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
@@ -3233,7 +3286,7 @@
     </row>
     <row r="122" spans="1:8">
       <c r="A122" s="14" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
@@ -3245,7 +3298,7 @@
     </row>
     <row r="123" spans="1:8">
       <c r="A123" s="14" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
@@ -3257,7 +3310,7 @@
     </row>
     <row r="124" spans="1:8">
       <c r="A124" s="14" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B124" s="15"/>
       <c r="C124" s="15"/>
@@ -3269,7 +3322,7 @@
     </row>
     <row r="125" spans="1:8">
       <c r="A125" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B125" s="15"/>
       <c r="C125" s="15"/>
@@ -3281,7 +3334,7 @@
     </row>
     <row r="126" spans="1:8">
       <c r="A126" s="14" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
@@ -3293,7 +3346,7 @@
     </row>
     <row r="127" spans="1:8">
       <c r="A127" s="14" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B127" s="15"/>
       <c r="C127" s="15"/>
@@ -3305,7 +3358,7 @@
     </row>
     <row r="128" spans="1:8">
       <c r="A128" s="14" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
@@ -3317,7 +3370,7 @@
     </row>
     <row r="129" spans="1:8">
       <c r="A129" s="14" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
@@ -3329,7 +3382,7 @@
     </row>
     <row r="130" spans="1:8">
       <c r="A130" s="14" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B130" s="15"/>
       <c r="C130" s="15"/>
@@ -3341,7 +3394,7 @@
     </row>
     <row r="131" spans="1:8">
       <c r="A131" s="14" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
@@ -3353,7 +3406,7 @@
     </row>
     <row r="132" spans="1:8">
       <c r="A132" s="14" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
@@ -3365,7 +3418,7 @@
     </row>
     <row r="133" spans="1:8">
       <c r="A133" s="14" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B133" s="15"/>
       <c r="C133" s="15"/>
@@ -3377,7 +3430,7 @@
     </row>
     <row r="134" spans="1:8">
       <c r="A134" s="14" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B134" s="15"/>
       <c r="C134" s="15"/>
@@ -3389,7 +3442,7 @@
     </row>
     <row r="135" spans="1:8">
       <c r="A135" s="14" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B135" s="15"/>
       <c r="C135" s="15"/>
@@ -3401,7 +3454,7 @@
     </row>
     <row r="136" spans="1:8">
       <c r="A136" s="14" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B136" s="15"/>
       <c r="C136" s="15"/>
@@ -3413,7 +3466,7 @@
     </row>
     <row r="137" ht="14.45" customHeight="1" spans="1:8">
       <c r="A137" s="11" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B137" s="12"/>
       <c r="C137" s="12"/>
@@ -3425,7 +3478,7 @@
     </row>
     <row r="138" spans="1:8">
       <c r="A138" s="14" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
@@ -3437,7 +3490,7 @@
     </row>
     <row r="139" spans="1:8">
       <c r="A139" s="14" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
@@ -3449,7 +3502,7 @@
     </row>
     <row r="140" spans="1:8">
       <c r="A140" s="14" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
@@ -3461,7 +3514,7 @@
     </row>
     <row r="141" spans="1:8">
       <c r="A141" s="14" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
@@ -3473,7 +3526,7 @@
     </row>
     <row r="142" spans="1:8">
       <c r="A142" s="14" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
@@ -3485,7 +3538,7 @@
     </row>
     <row r="143" spans="1:8">
       <c r="A143" s="14" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
@@ -3497,7 +3550,7 @@
     </row>
     <row r="144" spans="1:8">
       <c r="A144" s="14" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
@@ -3509,7 +3562,7 @@
     </row>
     <row r="145" spans="1:8">
       <c r="A145" s="14" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
@@ -3521,7 +3574,7 @@
     </row>
     <row r="146" spans="1:8">
       <c r="A146" s="14" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B146" s="15"/>
       <c r="C146" s="15"/>
@@ -3533,7 +3586,7 @@
     </row>
     <row r="147" spans="1:8">
       <c r="A147" s="14" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
@@ -3545,7 +3598,7 @@
     </row>
     <row r="148" spans="1:8">
       <c r="A148" s="14" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
@@ -3557,7 +3610,7 @@
     </row>
     <row r="149" spans="1:8">
       <c r="A149" s="14" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B149" s="15"/>
       <c r="C149" s="15"/>
@@ -3569,7 +3622,7 @@
     </row>
     <row r="150" spans="1:8">
       <c r="A150" s="14" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B150" s="15"/>
       <c r="C150" s="15"/>
@@ -3581,7 +3634,7 @@
     </row>
     <row r="151" spans="1:8">
       <c r="A151" s="14" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B151" s="15"/>
       <c r="C151" s="15"/>
@@ -3593,7 +3646,7 @@
     </row>
     <row r="152" spans="1:8">
       <c r="A152" s="14" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B152" s="15"/>
       <c r="C152" s="15"/>
@@ -3605,7 +3658,7 @@
     </row>
     <row r="153" spans="1:8">
       <c r="A153" s="14" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B153" s="15"/>
       <c r="C153" s="15"/>
@@ -3617,7 +3670,7 @@
     </row>
     <row r="154" spans="1:8">
       <c r="A154" s="14" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B154" s="15"/>
       <c r="C154" s="15"/>
@@ -3629,7 +3682,7 @@
     </row>
     <row r="155" spans="1:8">
       <c r="A155" s="14" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B155" s="15"/>
       <c r="C155" s="15"/>
@@ -3641,7 +3694,7 @@
     </row>
     <row r="156" spans="1:8">
       <c r="A156" s="14" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B156" s="15"/>
       <c r="C156" s="15"/>
@@ -3653,7 +3706,7 @@
     </row>
     <row r="157" spans="1:8">
       <c r="A157" s="14" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B157" s="15"/>
       <c r="C157" s="15"/>
@@ -3691,15 +3744,15 @@
   <sheetData>
     <row r="2" ht="17.4" spans="1:2">
       <c r="A2" s="3" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" ht="17.4" spans="1:2">
       <c r="A3" s="3" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B3" s="4"/>
     </row>
@@ -3709,19 +3762,19 @@
     </row>
     <row r="5" ht="17.4" spans="1:2">
       <c r="A5" s="6" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="B5" s="7"/>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="8" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="B6" s="9"/>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="8" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="B7" s="9"/>
     </row>
@@ -3738,1092 +3791,1092 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" s="11" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="13"/>
     </row>
     <row r="12" spans="1:3">
       <c r="A12" s="14" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B12" s="15"/>
       <c r="C12" s="15"/>
     </row>
     <row r="13" s="1" customFormat="1" spans="1:3">
       <c r="A13" s="14" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
     </row>
     <row r="14" s="1" customFormat="1" spans="1:3">
       <c r="A14" s="14" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B14" s="16"/>
       <c r="C14" s="16"/>
     </row>
     <row r="15" s="1" customFormat="1" spans="1:3">
       <c r="A15" s="14" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="B15" s="16"/>
       <c r="C15" s="16"/>
     </row>
     <row r="16" s="1" customFormat="1" spans="1:3">
       <c r="A16" s="14" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B16" s="16"/>
       <c r="C16" s="16"/>
     </row>
     <row r="17" s="1" customFormat="1" spans="1:3">
       <c r="A17" s="14" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B17" s="16"/>
       <c r="C17" s="16"/>
     </row>
     <row r="18" s="1" customFormat="1" spans="1:3">
       <c r="A18" s="14" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B18" s="16"/>
       <c r="C18" s="16"/>
     </row>
     <row r="19" s="1" customFormat="1" spans="1:3">
       <c r="A19" s="14" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
     </row>
     <row r="20" s="1" customFormat="1" spans="1:3">
       <c r="A20" s="14" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B20" s="16"/>
       <c r="C20" s="16"/>
     </row>
     <row r="21" s="1" customFormat="1" spans="1:3">
       <c r="A21" s="14" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="B21" s="16"/>
       <c r="C21" s="16"/>
     </row>
     <row r="22" s="1" customFormat="1" spans="1:3">
       <c r="A22" s="14" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B22" s="16"/>
       <c r="C22" s="16"/>
     </row>
     <row r="23" s="1" customFormat="1" spans="1:3">
       <c r="A23" s="14" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B23" s="16"/>
       <c r="C23" s="16"/>
     </row>
     <row r="24" s="1" customFormat="1" spans="1:3">
       <c r="A24" s="14" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B24" s="16"/>
       <c r="C24" s="16"/>
     </row>
     <row r="25" s="1" customFormat="1" spans="1:3">
       <c r="A25" s="14" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B25" s="16"/>
       <c r="C25" s="16"/>
     </row>
     <row r="26" s="1" customFormat="1" spans="1:3">
       <c r="A26" s="14" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B26" s="16"/>
       <c r="C26" s="16"/>
     </row>
     <row r="27" s="1" customFormat="1" spans="1:3">
       <c r="A27" s="14" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B27" s="16"/>
       <c r="C27" s="16"/>
     </row>
     <row r="28" s="1" customFormat="1" spans="1:3">
       <c r="A28" s="14" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B28" s="16"/>
       <c r="C28" s="16"/>
     </row>
     <row r="29" s="1" customFormat="1" spans="1:3">
       <c r="A29" s="14" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B29" s="16"/>
       <c r="C29" s="16"/>
     </row>
     <row r="30" s="1" customFormat="1" spans="1:3">
       <c r="A30" s="14" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B30" s="16"/>
       <c r="C30" s="16"/>
     </row>
     <row r="31" s="1" customFormat="1" spans="1:3">
       <c r="A31" s="14" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B31" s="16"/>
       <c r="C31" s="16"/>
     </row>
     <row r="32" s="1" customFormat="1" spans="1:3">
       <c r="A32" s="14" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B32" s="16"/>
       <c r="C32" s="16"/>
     </row>
     <row r="33" s="1" customFormat="1" spans="1:3">
       <c r="A33" s="14" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B33" s="16"/>
       <c r="C33" s="16"/>
     </row>
     <row r="34" s="1" customFormat="1" spans="1:3">
       <c r="A34" s="14" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B34" s="16"/>
       <c r="C34" s="16"/>
     </row>
     <row r="35" s="1" customFormat="1" spans="1:3">
       <c r="A35" s="14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B35" s="16"/>
       <c r="C35" s="16"/>
     </row>
     <row r="36" s="1" customFormat="1" spans="1:3">
       <c r="A36" s="14" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B36" s="16"/>
       <c r="C36" s="16"/>
     </row>
     <row r="37" s="1" customFormat="1" spans="1:3">
       <c r="A37" s="14" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B37" s="16"/>
       <c r="C37" s="16"/>
     </row>
     <row r="38" s="1" customFormat="1" spans="1:3">
       <c r="A38" s="14" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B38" s="16"/>
       <c r="C38" s="16"/>
     </row>
     <row r="39" s="1" customFormat="1" spans="1:3">
       <c r="A39" s="14" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B39" s="16"/>
       <c r="C39" s="16"/>
     </row>
     <row r="40" s="1" customFormat="1" spans="1:3">
       <c r="A40" s="14" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B40" s="16"/>
       <c r="C40" s="16"/>
     </row>
     <row r="41" s="1" customFormat="1" spans="1:3">
       <c r="A41" s="14" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="B41" s="16"/>
       <c r="C41" s="16"/>
     </row>
     <row r="42" s="1" customFormat="1" spans="1:3">
       <c r="A42" s="14" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="B42" s="16"/>
       <c r="C42" s="16"/>
     </row>
     <row r="43" s="1" customFormat="1" spans="1:3">
       <c r="A43" s="14" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="B43" s="16"/>
       <c r="C43" s="16"/>
     </row>
     <row r="44" s="1" customFormat="1" spans="1:3">
       <c r="A44" s="14" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="B44" s="16"/>
       <c r="C44" s="16"/>
     </row>
     <row r="45" s="1" customFormat="1" spans="1:3">
       <c r="A45" s="14" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="B45" s="16"/>
       <c r="C45" s="16"/>
     </row>
     <row r="46" s="1" customFormat="1" spans="1:3">
       <c r="A46" s="14" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B46" s="16"/>
       <c r="C46" s="16"/>
     </row>
     <row r="47" s="1" customFormat="1" spans="1:3">
       <c r="A47" s="14" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B47" s="16"/>
       <c r="C47" s="16"/>
     </row>
     <row r="48" s="1" customFormat="1" spans="1:3">
       <c r="A48" s="14" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B48" s="16"/>
       <c r="C48" s="16"/>
     </row>
     <row r="49" s="1" customFormat="1" spans="1:3">
       <c r="A49" s="14" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B49" s="16"/>
       <c r="C49" s="16"/>
     </row>
     <row r="50" s="1" customFormat="1" spans="1:3">
       <c r="A50" s="14" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B50" s="16"/>
       <c r="C50" s="16"/>
     </row>
     <row r="51" s="1" customFormat="1" spans="1:3">
       <c r="A51" s="14" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B51" s="16"/>
       <c r="C51" s="16"/>
     </row>
     <row r="52" s="1" customFormat="1" spans="1:3">
       <c r="A52" s="14" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B52" s="16"/>
       <c r="C52" s="16"/>
     </row>
     <row r="53" s="1" customFormat="1" spans="1:3">
       <c r="A53" s="14" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B53" s="16"/>
       <c r="C53" s="16"/>
     </row>
     <row r="54" s="1" customFormat="1" spans="1:3">
       <c r="A54" s="14" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B54" s="16"/>
       <c r="C54" s="16"/>
     </row>
     <row r="55" s="1" customFormat="1" spans="1:3">
       <c r="A55" s="14" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B55" s="16"/>
       <c r="C55" s="16"/>
     </row>
     <row r="56" s="1" customFormat="1" spans="1:3">
       <c r="A56" s="14" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B56" s="16"/>
       <c r="C56" s="16"/>
     </row>
     <row r="57" s="1" customFormat="1" spans="1:3">
       <c r="A57" s="14" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="B57" s="16"/>
       <c r="C57" s="16"/>
     </row>
     <row r="58" s="1" customFormat="1" spans="1:3">
       <c r="A58" s="14" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B58" s="16"/>
       <c r="C58" s="16"/>
     </row>
     <row r="59" s="1" customFormat="1" spans="1:3">
       <c r="A59" s="14" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B59" s="16"/>
       <c r="C59" s="16"/>
     </row>
     <row r="60" s="1" customFormat="1" spans="1:3">
       <c r="A60" s="14" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="B60" s="16"/>
       <c r="C60" s="16"/>
     </row>
     <row r="61" s="1" customFormat="1" spans="1:3">
       <c r="A61" s="14" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B61" s="16"/>
       <c r="C61" s="16"/>
     </row>
     <row r="62" s="2" customFormat="1" spans="1:3">
       <c r="A62" s="11" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B62" s="12"/>
       <c r="C62" s="13"/>
     </row>
     <row r="63" s="1" customFormat="1" spans="1:3">
       <c r="A63" s="17" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="B63" s="16"/>
       <c r="C63" s="16"/>
     </row>
     <row r="64" s="1" customFormat="1" spans="1:3">
       <c r="A64" s="17" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="B64" s="16"/>
       <c r="C64" s="16"/>
     </row>
     <row r="65" s="1" customFormat="1" spans="1:3">
       <c r="A65" s="17" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B65" s="16"/>
       <c r="C65" s="16"/>
     </row>
     <row r="66" s="1" customFormat="1" spans="1:3">
       <c r="A66" s="17" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B66" s="16"/>
       <c r="C66" s="16"/>
     </row>
     <row r="67" s="1" customFormat="1" spans="1:3">
       <c r="A67" s="17" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="B67" s="16"/>
       <c r="C67" s="16"/>
     </row>
     <row r="68" s="1" customFormat="1" spans="1:3">
       <c r="A68" s="17" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B68" s="16"/>
       <c r="C68" s="16"/>
     </row>
     <row r="69" s="1" customFormat="1" spans="1:3">
       <c r="A69" s="17" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B69" s="16"/>
       <c r="C69" s="16"/>
     </row>
     <row r="70" s="1" customFormat="1" spans="1:3">
       <c r="A70" s="17" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B70" s="16"/>
       <c r="C70" s="16"/>
     </row>
     <row r="71" s="1" customFormat="1" spans="1:3">
       <c r="A71" s="17" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B71" s="16"/>
       <c r="C71" s="16"/>
     </row>
     <row r="72" s="1" customFormat="1" spans="1:3">
       <c r="A72" s="17" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="B72" s="16"/>
       <c r="C72" s="16"/>
     </row>
     <row r="73" s="1" customFormat="1" spans="1:3">
       <c r="A73" s="17" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B73" s="16"/>
       <c r="C73" s="16"/>
     </row>
     <row r="74" s="1" customFormat="1" spans="1:3">
       <c r="A74" s="17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="B74" s="16"/>
       <c r="C74" s="16"/>
     </row>
     <row r="75" s="1" customFormat="1" spans="1:3">
       <c r="A75" s="17" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B75" s="16"/>
       <c r="C75" s="16"/>
     </row>
     <row r="76" s="1" customFormat="1" spans="1:3">
       <c r="A76" s="17" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="B76" s="16"/>
       <c r="C76" s="16"/>
     </row>
     <row r="77" s="1" customFormat="1" spans="1:3">
       <c r="A77" s="17" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="B77" s="16"/>
       <c r="C77" s="16"/>
     </row>
     <row r="78" s="1" customFormat="1" spans="1:3">
       <c r="A78" s="17" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B78" s="16"/>
       <c r="C78" s="16"/>
     </row>
     <row r="79" s="1" customFormat="1" spans="1:3">
       <c r="A79" s="17" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="B79" s="16"/>
       <c r="C79" s="16"/>
     </row>
     <row r="80" s="1" customFormat="1" spans="1:3">
       <c r="A80" s="17" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="B80" s="16"/>
       <c r="C80" s="16"/>
     </row>
     <row r="81" s="1" customFormat="1" spans="1:3">
       <c r="A81" s="17" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B81" s="16"/>
       <c r="C81" s="16"/>
     </row>
     <row r="82" s="1" customFormat="1" spans="1:3">
       <c r="A82" s="17" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="B82" s="16"/>
       <c r="C82" s="16"/>
     </row>
     <row r="83" s="2" customFormat="1" spans="1:3">
       <c r="A83" s="11" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B83" s="12"/>
       <c r="C83" s="13"/>
     </row>
     <row r="84" s="1" customFormat="1" spans="1:3">
       <c r="A84" s="18" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B84" s="18"/>
       <c r="C84" s="18"/>
     </row>
     <row r="85" s="1" customFormat="1" spans="1:3">
       <c r="A85" s="18" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="B85" s="2"/>
       <c r="C85" s="18"/>
     </row>
     <row r="86" s="1" customFormat="1" spans="1:3">
       <c r="A86" s="18" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B86" s="16"/>
       <c r="C86" s="18"/>
     </row>
     <row r="87" s="1" customFormat="1" spans="1:3">
       <c r="A87" s="18" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B87" s="2"/>
       <c r="C87" s="18"/>
     </row>
     <row r="88" s="1" customFormat="1" spans="1:3">
       <c r="A88" s="18" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B88" s="16"/>
       <c r="C88" s="18"/>
     </row>
     <row r="89" s="1" customFormat="1" spans="1:3">
       <c r="A89" s="18" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B89" s="15"/>
       <c r="C89" s="18"/>
     </row>
     <row r="90" s="1" customFormat="1" spans="1:3">
       <c r="A90" s="18" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B90" s="15"/>
       <c r="C90" s="18"/>
     </row>
     <row r="91" s="1" customFormat="1" spans="1:3">
       <c r="A91" s="18" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B91" s="15"/>
       <c r="C91" s="18"/>
     </row>
     <row r="92" s="1" customFormat="1" spans="1:3">
       <c r="A92" s="18" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B92" s="15"/>
       <c r="C92" s="18"/>
     </row>
     <row r="93" s="1" customFormat="1" spans="1:3">
       <c r="A93" s="18" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B93" s="15"/>
       <c r="C93" s="18"/>
     </row>
     <row r="94" s="1" customFormat="1" spans="1:3">
       <c r="A94" s="18" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B94" s="15"/>
       <c r="C94" s="18"/>
     </row>
     <row r="95" s="1" customFormat="1" spans="1:3">
       <c r="A95" s="18" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B95" s="15"/>
       <c r="C95" s="18"/>
     </row>
     <row r="96" s="1" customFormat="1" spans="1:3">
       <c r="A96" s="18" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B96" s="15"/>
       <c r="C96" s="18"/>
     </row>
     <row r="97" s="1" customFormat="1" spans="1:3">
       <c r="A97" s="18" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B97" s="15"/>
       <c r="C97" s="18"/>
     </row>
     <row r="98" s="1" customFormat="1" spans="1:3">
       <c r="A98" s="18" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B98" s="15"/>
       <c r="C98" s="18"/>
     </row>
     <row r="99" s="1" customFormat="1" spans="1:3">
       <c r="A99" s="18" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B99" s="15"/>
       <c r="C99" s="18"/>
     </row>
     <row r="100" s="1" customFormat="1" spans="1:3">
       <c r="A100" s="18" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B100" s="15"/>
       <c r="C100" s="18"/>
     </row>
     <row r="101" s="1" customFormat="1" spans="1:3">
       <c r="A101" s="18" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B101" s="15"/>
       <c r="C101" s="18"/>
     </row>
     <row r="102" s="1" customFormat="1" spans="1:3">
       <c r="A102" s="18" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B102" s="15"/>
       <c r="C102" s="18"/>
     </row>
     <row r="103" s="1" customFormat="1" spans="1:3">
       <c r="A103" s="18" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B103" s="15"/>
       <c r="C103" s="18"/>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" s="11" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B104" s="12"/>
       <c r="C104" s="13"/>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B105" s="15"/>
       <c r="C105" s="15"/>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" s="14" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B106" s="15"/>
       <c r="C106" s="15"/>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" s="14" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B107" s="15"/>
       <c r="C107" s="15"/>
     </row>
     <row r="108" spans="1:3">
       <c r="A108" s="14" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B108" s="15"/>
       <c r="C108" s="15"/>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" s="14" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B109" s="15"/>
       <c r="C109" s="15"/>
     </row>
     <row r="110" spans="1:3">
       <c r="A110" s="14" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B110" s="15"/>
       <c r="C110" s="15"/>
     </row>
     <row r="111" spans="1:3">
       <c r="A111" s="14" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B111" s="15"/>
       <c r="C111" s="15"/>
     </row>
     <row r="112" spans="1:3">
       <c r="A112" s="14" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B112" s="15"/>
       <c r="C112" s="15"/>
     </row>
     <row r="113" spans="1:3">
       <c r="A113" s="14" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B113" s="15"/>
       <c r="C113" s="15"/>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" s="14" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B114" s="15"/>
       <c r="C114" s="15"/>
     </row>
     <row r="115" spans="1:3">
       <c r="A115" s="14" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="B115" s="15"/>
       <c r="C115" s="15"/>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B116" s="15"/>
       <c r="C116" s="15"/>
     </row>
     <row r="117" spans="1:3">
       <c r="A117" s="14" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B117" s="15"/>
       <c r="C117" s="15"/>
     </row>
     <row r="118" spans="1:3">
       <c r="A118" s="14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="B118" s="15"/>
       <c r="C118" s="15"/>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" s="14" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B119" s="15"/>
       <c r="C119" s="15"/>
     </row>
     <row r="120" spans="1:3">
       <c r="A120" s="14" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B120" s="15"/>
       <c r="C120" s="15"/>
     </row>
     <row r="121" spans="1:3">
       <c r="A121" s="14" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="B121" s="15"/>
       <c r="C121" s="15"/>
     </row>
     <row r="122" spans="1:3">
       <c r="A122" s="14" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B122" s="15"/>
       <c r="C122" s="15"/>
     </row>
     <row r="123" spans="1:3">
       <c r="A123" s="14" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B123" s="15"/>
       <c r="C123" s="15"/>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" s="14" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B124" s="15"/>
       <c r="C124" s="15"/>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" s="11" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="B125" s="12"/>
       <c r="C125" s="13"/>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" s="14" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="B126" s="15"/>
       <c r="C126" s="15"/>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" s="14" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B127" s="15"/>
       <c r="C127" s="15"/>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" s="14" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="B128" s="15"/>
       <c r="C128" s="15"/>
     </row>
     <row r="129" spans="1:3">
       <c r="A129" s="14" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="B129" s="15"/>
       <c r="C129" s="15"/>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" s="14" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B130" s="15"/>
       <c r="C130" s="15"/>
     </row>
     <row r="131" spans="1:3">
       <c r="A131" s="14" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="B131" s="15"/>
       <c r="C131" s="15"/>
     </row>
     <row r="132" spans="1:3">
       <c r="A132" s="14" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="B132" s="15"/>
       <c r="C132" s="15"/>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" s="14" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B133" s="15"/>
       <c r="C133" s="15"/>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B134" s="15"/>
       <c r="C134" s="15"/>
     </row>
     <row r="135" spans="1:3">
       <c r="A135" s="14" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B135" s="15"/>
       <c r="C135" s="15"/>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" s="14" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="B136" s="15"/>
       <c r="C136" s="15"/>
     </row>
     <row r="137" spans="1:3">
       <c r="A137" s="14" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B137" s="15"/>
       <c r="C137" s="15"/>
     </row>
     <row r="138" spans="1:3">
       <c r="A138" s="14" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="B138" s="15"/>
       <c r="C138" s="15"/>
     </row>
     <row r="139" spans="1:3">
       <c r="A139" s="14" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="B139" s="15"/>
       <c r="C139" s="15"/>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" s="14" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="B140" s="15"/>
       <c r="C140" s="15"/>
     </row>
     <row r="141" spans="1:3">
       <c r="A141" s="14" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B141" s="15"/>
       <c r="C141" s="15"/>
     </row>
     <row r="142" spans="1:3">
       <c r="A142" s="14" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="B142" s="15"/>
       <c r="C142" s="15"/>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" s="14" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="B143" s="15"/>
       <c r="C143" s="15"/>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" s="14" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B144" s="15"/>
       <c r="C144" s="15"/>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" s="14" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="B145" s="15"/>
       <c r="C145" s="15"/>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" s="11" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="B146" s="12"/>
       <c r="C146" s="13"/>
     </row>
     <row r="147" spans="1:3">
       <c r="A147" s="14" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="B147" s="15"/>
       <c r="C147" s="15"/>
     </row>
     <row r="148" spans="1:3">
       <c r="A148" s="14" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B148" s="15"/>
       <c r="C148" s="15"/>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" s="14" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="B149" s="15"/>
       <c r="C149" s="15"/>
     </row>
     <row r="150" spans="1:3">
       <c r="A150" s="14" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B150" s="15"/>
       <c r="C150" s="15"/>
     </row>
     <row r="151" spans="1:3">
       <c r="A151" s="14" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="B151" s="15"/>
       <c r="C151" s="15"/>
     </row>
     <row r="152" spans="1:3">
       <c r="A152" s="14" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="B152" s="15"/>
       <c r="C152" s="15"/>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" s="14" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="B153" s="15"/>
       <c r="C153" s="15"/>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" s="14" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="B154" s="15"/>
       <c r="C154" s="15"/>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" s="14" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B155" s="15"/>
       <c r="C155" s="15"/>
     </row>
     <row r="156" spans="1:3">
       <c r="A156" s="14" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="B156" s="15"/>
       <c r="C156" s="15"/>
     </row>
     <row r="157" spans="1:3">
       <c r="A157" s="14" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="B157" s="15"/>
       <c r="C157" s="15"/>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" s="14" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="B158" s="15"/>
       <c r="C158" s="15"/>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" s="14" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="B159" s="15"/>
       <c r="C159" s="15"/>
     </row>
     <row r="160" spans="1:3">
       <c r="A160" s="14" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="B160" s="15"/>
       <c r="C160" s="15"/>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" s="14" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="B161" s="15"/>
       <c r="C161" s="15"/>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" s="14" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B162" s="15"/>
       <c r="C162" s="15"/>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" s="14" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="B163" s="15"/>
       <c r="C163" s="15"/>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" s="14" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="B164" s="15"/>
       <c r="C164" s="15"/>
     </row>
     <row r="165" spans="1:3">
       <c r="A165" s="14" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="B165" s="15"/>
       <c r="C165" s="15"/>
     </row>
     <row r="166" spans="1:3">
       <c r="A166" s="14" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="B166" s="15"/>
       <c r="C166" s="15"/>

</xml_diff>